<commit_message>
docs+data: Marzo=BlackBerry se añade como mes fijo
Igual que Octubre=Original y Diciembre=Winter, Marzo siempre usa la
plantilla BlackBerry y no se puede mover con la mecánica de
intercambio. Actualiza CLAUDE.md y SPEC.md (los ejemplos de swap que
usaban Marzo como destino ahora usan Abril), y el Excel real
(Calendario_Sabores + Instrucciones) para que quede consistente.

No hace falta tocar código: apply_override_swap() ya decide qué mes es
fijo a partir del dato (columna Tipo / CalendarEntry.fijo), no de una
lista hardcodeada.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos_carteles_oncle_jack.xlsx
+++ b/datos_carteles_oncle_jack.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sabores_disponibles" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendario_Sabores" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Eventos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sabores_disponibles" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Calendario_Sabores" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Eventos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -509,21 +509,21 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2. 'Calendario_Sabores': qué sabor le toca a cada mes de la temporada 26/27. Octubre siempre es 'Original'</t>
+          <t>2. 'Calendario_Sabores': qué sabor le toca a cada mes de la temporada 26/27. Octubre siempre es 'Original',</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   y Diciembre siempre es 'Winter' — esas dos filas no se tocan. El resto de meses hay que rellenarlos</t>
+          <t xml:space="preserve">   Diciembre siempre es 'Winter' y Marzo siempre es 'BlackBerry' — esas tres filas no se tocan. El resto de meses</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">   con el sabor que prefieras (sin repetir), eligiendo de los que quedan en 'Sabores_disponibles'.</t>
+          <t xml:space="preserve">   hay que rellenarlos con el sabor que prefieras (sin repetir), eligiendo de los que quedan en 'Sabores_disponibles'.</t>
         </is>
       </c>
     </row>
@@ -833,10 +833,14 @@
           <t>Marzo</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>BlackBerry</t>
+        </is>
+      </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>Fijo — no cambiar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: Excel real con URLs de Canva y Comico_2_Nombre (editado por el usuario)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos_carteles_oncle_jack.xlsx
+++ b/datos_carteles_oncle_jack.xlsx
@@ -211,28 +211,28 @@
     <t xml:space="preserve">Sergio Afonso</t>
   </si>
   <si>
-    <t xml:space="preserve">Nombre Cómico 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/uc?id=EJEMPLO1</t>
+    <t xml:space="preserve">Ikki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://canva.link/pq2xdlk9xlfndse</t>
   </si>
   <si>
     <t xml:space="preserve">Santi Rou</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/uc?id=EJEMPLO2</t>
+    <t xml:space="preserve">https://canva.link/dp9qaoq07n1l6b2</t>
   </si>
   <si>
     <t xml:space="preserve">Fiorella</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/uc?id=EJEMPLO3</t>
+    <t xml:space="preserve">https://canva.link/kd98shpetaj2am1</t>
   </si>
   <si>
     <t xml:space="preserve">Bad Funny</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/uc?id=EJEMPLO4</t>
+    <t xml:space="preserve">https://canva.link/zyxvd0tfeqmde4l</t>
   </si>
   <si>
     <t xml:space="preserve">Pendiente</t>
@@ -264,7 +264,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -324,18 +324,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF7A5C00"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
       <i val="true"/>
       <sz val="10"/>
       <color rgb="FF7A5C00"/>
@@ -349,6 +337,7 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -416,55 +405,55 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -723,110 +712,110 @@
   <dimension ref="A1:A22"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="105"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="105"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
+      <c r="A2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
+      <c r="A12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2"/>
+      <c r="A20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>18</v>
       </c>
     </row>
@@ -849,66 +838,66 @@
   <dimension ref="A1:A12"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>30</v>
       </c>
     </row>
@@ -931,116 +920,116 @@
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="1" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1063,53 +1052,53 @@
   <dimension ref="A1:O13"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="1" style="1" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="5" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1210,6 +1199,12 @@
       <c r="A13" s="13"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1" display="https://canva.link/pq2xdlk9xlfndse"/>
+    <hyperlink ref="H2" r:id="rId2" display="https://canva.link/dp9qaoq07n1l6b2"/>
+    <hyperlink ref="J2" r:id="rId3" display="https://canva.link/kd98shpetaj2am1"/>
+    <hyperlink ref="L2" r:id="rId4" display="https://canva.link/zyxvd0tfeqmde4l"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
feat: validate_foto_url (tarea 15, SPEC 5.5) (#1)
* docs: SPEC 5.5 (fotos Canva) y backlog tareas 15-18

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* data: Excel real con URLs de Canva y Comico_2_Nombre (editado por el usuario)

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* feat: validate_foto_url (tarea 15, SPEC 5.5)

- foto_url.py: módulo para validar URLs de fotos de Canva
- tests/test_foto_url.py: suite de tests (TDD)

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos_carteles_oncle_jack.xlsx
+++ b/datos_carteles_oncle_jack.xlsx
@@ -211,28 +211,28 @@
     <t xml:space="preserve">Sergio Afonso</t>
   </si>
   <si>
-    <t xml:space="preserve">Nombre Cómico 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://drive.google.com/uc?id=EJEMPLO1</t>
+    <t xml:space="preserve">Ikki</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://canva.link/pq2xdlk9xlfndse</t>
   </si>
   <si>
     <t xml:space="preserve">Santi Rou</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/uc?id=EJEMPLO2</t>
+    <t xml:space="preserve">https://canva.link/dp9qaoq07n1l6b2</t>
   </si>
   <si>
     <t xml:space="preserve">Fiorella</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/uc?id=EJEMPLO3</t>
+    <t xml:space="preserve">https://canva.link/kd98shpetaj2am1</t>
   </si>
   <si>
     <t xml:space="preserve">Bad Funny</t>
   </si>
   <si>
-    <t xml:space="preserve">https://drive.google.com/uc?id=EJEMPLO4</t>
+    <t xml:space="preserve">https://canva.link/zyxvd0tfeqmde4l</t>
   </si>
   <si>
     <t xml:space="preserve">Pendiente</t>
@@ -264,7 +264,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -324,18 +324,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF7A5C00"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
       <i val="true"/>
       <sz val="10"/>
       <color rgb="FF7A5C00"/>
@@ -349,6 +337,7 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -416,55 +405,55 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -723,110 +712,110 @@
   <dimension ref="A1:A22"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="105"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="105"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
+      <c r="A2" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2"/>
+      <c r="A12" s="3"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2"/>
+      <c r="A20" s="3"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
+      <c r="A21" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>18</v>
       </c>
     </row>
@@ -849,66 +838,66 @@
   <dimension ref="A1:A12"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>30</v>
       </c>
     </row>
@@ -931,116 +920,116 @@
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="1" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1063,53 +1052,53 @@
   <dimension ref="A1:O13"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="1" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="1" style="1" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>49</v>
       </c>
       <c r="G1" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="N1" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="O1" s="5" t="s">
         <v>58</v>
       </c>
     </row>
@@ -1210,6 +1199,12 @@
       <c r="A13" s="13"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F2" r:id="rId1" display="https://canva.link/pq2xdlk9xlfndse"/>
+    <hyperlink ref="H2" r:id="rId2" display="https://canva.link/dp9qaoq07n1l6b2"/>
+    <hyperlink ref="J2" r:id="rId3" display="https://canva.link/kd98shpetaj2am1"/>
+    <hyperlink ref="L2" r:id="rId4" display="https://canva.link/zyxvd0tfeqmde4l"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>